<commit_message>
Updated erroneous file names
</commit_message>
<xml_diff>
--- a/musicCraft/musicCodex.xlsx
+++ b/musicCraft/musicCodex.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\swamp\minecraft\swampCraft\musicCraft\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{56AC25AE-560E-43EA-82A0-D5EF0C60F522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E225E67B-90DF-4301-853D-A0F538E5026D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32460" yWindow="600" windowWidth="38370" windowHeight="20520" firstSheet="12" activeTab="18" xr2:uid="{72A73C0B-CC92-450B-BE01-D1BF5D132B64}"/>
+    <workbookView xWindow="32460" yWindow="600" windowWidth="38370" windowHeight="20520" firstSheet="5" activeTab="7" xr2:uid="{72A73C0B-CC92-450B-BE01-D1BF5D132B64}"/>
   </bookViews>
   <sheets>
     <sheet name="Tool - 10,000 Days" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
     <sheet name="Muse - Black Holes &amp; Revelation" sheetId="16" r:id="rId16"/>
     <sheet name="Muse - The 2nd Law" sheetId="17" r:id="rId17"/>
     <sheet name="Muse - The Resistance" sheetId="18" r:id="rId18"/>
-    <sheet name="Muse - Will of the People" sheetId="19" r:id="rId19"/>
+    <sheet name="musicCodex" sheetId="19" r:id="rId19"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="584">
   <si>
     <t>Vicarious</t>
   </si>
@@ -1803,6 +1803,9 @@
   </si>
   <si>
     <t>You Make Me Feel Like It's Halloween.dfpwm</t>
+  </si>
+  <si>
+    <t>Random Access Memories</t>
   </si>
 </sst>
 </file>
@@ -5702,7 +5705,7 @@
         <v>179</v>
       </c>
       <c r="B2" t="s">
-        <v>180</v>
+        <v>583</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>210</v>

</xml_diff>